<commit_message>
Refine report equations, dated citations and procurement scope
</commit_message>
<xml_diff>
--- a/deliverables/assignment1_models.xlsx
+++ b/deliverables/assignment1_models.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="273">
   <si>
     <t>Assignment 1 | Model guide and scope</t>
   </si>
@@ -74,7 +74,7 @@
     <t>Sensitivity varies only Google subscription price and Exchange FTE at USD 80,000/FTE/year. A USD 14 plan is a cost stress, not an assertion of equal plan features.</t>
   </si>
   <si>
-    <t>Sources contains exact URLs, supported claims and verification status. Official Google pages and Microsoft Learn sources were checked. The Microsoft licensing commercial page still returned HTTP 403 and needs manual review. Model budgets are not vendor quotations.</t>
+    <t>Sources maps the official documentation to specific claims and records publication/revision dates. Licensing, staffing and hardware inputs are planning assumptions; procurement requires current entitlements and comparable quotations.</t>
   </si>
   <si>
     <t>Readiness: see Checks. Cached values are included; open in Excel/LibreOffice to recalculate after changing inputs. External PNG/PDF/SVG figures represent the original baseline and do not auto-refresh.</t>
@@ -383,7 +383,7 @@
     <t>Alternative timing LTV</t>
   </si>
   <si>
-    <t>Base formula: Σ[t=1..5] GP×(1−risk loss)×(1−annual churn)^(t−1)/(1+discount)^t. Alternative timing applies churn before every year’s contribution, including year 1. Neither is a perpetual LTV.</t>
+    <t>The report presents the formal LTV equation. This sheet sums five discounted annual contributions, weighted by start-year survival. Alternative timing requires survival through year 1; neither convention includes a terminal value.</t>
   </si>
   <si>
     <t>Funding credit changes the cost assigned to the focal product, not total ecosystem resource use. This is a transparent hypothetical cross-subsidy mechanism, not observed Google or Microsoft financial performance.</t>
@@ -536,6 +536,9 @@
     <t>Official GitHub source</t>
   </si>
   <si>
+    <t>Citation date basis</t>
+  </si>
+  <si>
     <t>G1</t>
   </si>
   <si>
@@ -554,10 +557,13 @@
     <t>VERIFIED: original official announcement retrieved; dated 28 August 2006.</t>
   </si>
   <si>
+    <t>2006-08-28 — Date displayed on the original announcement</t>
+  </si>
+  <si>
     <t>G2</t>
   </si>
   <si>
-    <t>Google (n.d.-a)</t>
+    <t>Google (n.d.)</t>
   </si>
   <si>
     <t>Google Workspace pricing</t>
@@ -566,16 +572,19 @@
     <t>https://workspace.google.com/pricing.html</t>
   </si>
   <si>
-    <t>Product/bundle and current plan/commitment checks only. USD 7 and 14 are scenario inputs, not verified quotes.</t>
+    <t>Current suite scope and annual-commitment price context; flat five-year USD 7/14 inputs remain illustrative assumptions.</t>
   </si>
   <si>
     <t>VERIFIED: official pricing page retrieved. Annual-commitment standard USD 7/14 displayed, with separate promotions; five-year flat prices remain assumptions.</t>
   </si>
   <si>
+    <t>Undated — No publication/revision date displayed</t>
+  </si>
+  <si>
     <t>G3</t>
   </si>
   <si>
-    <t>Google (n.d.-b)</t>
+    <t>Google (2025)</t>
   </si>
   <si>
     <t>Google Workspace Marketplace</t>
@@ -590,10 +599,13 @@
     <t>VERIFIED: official Marketplace overview retrieved; third-party apps and add-on publishing documented.</t>
   </si>
   <si>
+    <t>2025-09-26 — Displayed last-updated date</t>
+  </si>
+  <si>
     <t>G4</t>
   </si>
   <si>
-    <t>Google (n.d.-c)</t>
+    <t>Google (2026b)</t>
   </si>
   <si>
     <t>Gmail API: Python quickstart</t>
@@ -611,10 +623,13 @@
     <t>https://raw.githubusercontent.com/googleworkspace/python-samples/main/gmail/quickstart/quickstart.py</t>
   </si>
   <si>
+    <t>2026-10-12 — Displayed last-updated date</t>
+  </si>
+  <si>
     <t>G5</t>
   </si>
   <si>
-    <t>Google (n.d.-d)</t>
+    <t>Google (2026a)</t>
   </si>
   <si>
     <t>Admin SDK Directory API: Python quickstart</t>
@@ -632,7 +647,7 @@
     <t>G6</t>
   </si>
   <si>
-    <t>Google (n.d.-e)</t>
+    <t>Google (2026c)</t>
   </si>
   <si>
     <t>Google Drive API: Python quickstart</t>
@@ -647,28 +662,10 @@
     <t>https://raw.githubusercontent.com/googleworkspace/python-samples/main/drive/quickstart/quickstart.py</t>
   </si>
   <si>
-    <t>M1</t>
-  </si>
-  <si>
-    <t>Microsoft (n.d.-a)</t>
-  </si>
-  <si>
-    <t>Exchange Server licensing overview</t>
-  </si>
-  <si>
-    <t>https://www.microsoft.com/en-us/microsoft-365/exchange/microsoft-exchange-server-licensing-licensing-overview</t>
-  </si>
-  <si>
-    <t>Licensing due diligence only. USD 12,000/year is an illustrative allowance, not a vendor quotation.</t>
-  </si>
-  <si>
-    <t>PENDING: commercial page returned HTTP 403 after network restoration. SE entitlements and underlying Windows/CAL coverage need a current quote; no price or exact entitlement claim is used.</t>
-  </si>
-  <si>
     <t>M2</t>
   </si>
   <si>
-    <t>Microsoft (n.d.-b)</t>
+    <t>Microsoft (2026a)</t>
   </si>
   <si>
     <t>New-Mailbox (ExchangePowerShell)</t>
@@ -680,16 +677,19 @@
     <t>Official applicability lists both Exchange Server SE and Exchange Online; mailbox and user-account creation.</t>
   </si>
   <si>
-    <t>VERIFIED: official MicrosoftDocs source retrieved; rendered Learn page not accessed.</t>
+    <t>Official Microsoft Learn page and MicrosoftDocs source reviewed.</t>
   </si>
   <si>
     <t>https://raw.githubusercontent.com/MicrosoftDocs/office-docs-powershell/main/exchange/exchange-ps/ExchangePowerShell/New-Mailbox.md</t>
   </si>
   <si>
+    <t>2026-05-16 — Revision date in official page updated_at metadata</t>
+  </si>
+  <si>
     <t>M3</t>
   </si>
   <si>
-    <t>Microsoft (n.d.-c)</t>
+    <t>Microsoft (2026b)</t>
   </si>
   <si>
     <t>New-MigrationBatch (ExchangePowerShell)</t>
@@ -704,10 +704,13 @@
     <t>https://raw.githubusercontent.com/MicrosoftDocs/office-docs-powershell/main/exchange/exchange-ps/ExchangePowerShell/New-MigrationBatch.md</t>
   </si>
   <si>
+    <t>2026-05-28 — Revision date in official page updated_at metadata</t>
+  </si>
+  <si>
     <t>M4</t>
   </si>
   <si>
-    <t>Microsoft (n.d.-d)</t>
+    <t>Microsoft (2025a)</t>
   </si>
   <si>
     <t>Exchange Online service description</t>
@@ -719,13 +722,16 @@
     <t>Exchange Online as the procurement comparator; current price/features not asserted.</t>
   </si>
   <si>
-    <t>VERIFIED: official Learn service description retrieved. Commercial pricing page returned HTTP 403; no Exchange Online price is modeled.</t>
+    <t>Official Microsoft Learn service description reviewed; Exchange Online price is outside the quantified scenario.</t>
+  </si>
+  <si>
+    <t>2025-12-09 — Displayed last-updated date</t>
   </si>
   <si>
     <t>M5</t>
   </si>
   <si>
-    <t>Microsoft (n.d.-e)</t>
+    <t>Microsoft (2025b)</t>
   </si>
   <si>
     <t>Exchange Server architecture</t>
@@ -734,16 +740,19 @@
     <t>https://learn.microsoft.com/en-us/exchange/architecture/architecture?view=exchserver-2019</t>
   </si>
   <si>
-    <t>Server-side architecture and deployment responsibilities; SE applicability requires checking.</t>
+    <t>Exchange Mailbox server architecture and administration; the page applies to Subscription Edition.</t>
   </si>
   <si>
     <t>VERIFIED: official Learn architecture page retrieved; current page applies to Subscription Edition.</t>
   </si>
   <si>
+    <t>2025-04-02 — Displayed last-updated date</t>
+  </si>
+  <si>
     <t>M6</t>
   </si>
   <si>
-    <t>Microsoft (n.d.-f)</t>
+    <t>Microsoft (2025c)</t>
   </si>
   <si>
     <t>What is new in Exchange Server Subscription Edition (SE)</t>
@@ -756,6 +765,9 @@
   </si>
   <si>
     <t>VERIFIED: official Learn SE page retrieved; no retirement or release-date assertion used.</t>
+  </si>
+  <si>
+    <t>2025-06-16 — Displayed last-updated date</t>
   </si>
   <si>
     <t>Access audit date: 16 October 2026. A verified GitHub sample supports only the stated API/documentation claim. It is not a live API test, a product-price verification or evidence of vendor churn/CAC.</t>
@@ -1012,7 +1024,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>2026–2030 scenarios: c(n)=0.18 exp(−0.10n)</a:t>
+              <a:t>Annual churn by integration count | 2026–2030 scenarios</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -3738,8 +3750,7 @@
     <col min="1" max="1" width="8.7109375" customWidth="1"/>
     <col min="2" max="2" width="22.7109375" customWidth="1"/>
     <col min="3" max="3" width="35.7109375" customWidth="1"/>
-    <col min="4" max="7" width="52.7109375" customWidth="1"/>
-    <col min="8" max="8" width="19.7109375" customWidth="1"/>
+    <col min="4" max="8" width="52.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="22" customHeight="1">
@@ -3776,272 +3787,287 @@
       <c r="G3" s="3" t="s">
         <v>162</v>
       </c>
+      <c r="H3" s="3" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="95" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G4" s="4"/>
+      <c r="H4" s="4" t="s">
+        <v>170</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="95" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G5" s="4"/>
+      <c r="H5" s="4" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="95" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="G6" s="4"/>
+      <c r="H6" s="4" t="s">
+        <v>184</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="95" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>187</v>
+        <v>191</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="95" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="E8" s="4" t="s">
+      <c r="G8" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="H8" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="95" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>199</v>
+        <v>204</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="95" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="G10" s="4"/>
+        <v>210</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>212</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="95" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="E11" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="F11" s="4" t="s">
-        <v>211</v>
-      </c>
       <c r="G11" s="4" t="s">
-        <v>212</v>
+        <v>218</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="95" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>218</v>
+        <v>225</v>
+      </c>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="95" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="G13" s="4"/>
+      <c r="H13" s="4" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="95" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="G14" s="4"/>
-    </row>
-    <row r="15" spans="1:8" ht="95" customHeight="1">
-      <c r="A15" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="G15" s="4"/>
+      <c r="H14" s="4" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="19" spans="1:8" ht="25" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -4077,13 +4103,12 @@
     <hyperlink ref="D9" r:id="rId8"/>
     <hyperlink ref="G9" r:id="rId9"/>
     <hyperlink ref="D10" r:id="rId10"/>
-    <hyperlink ref="D11" r:id="rId11"/>
-    <hyperlink ref="G11" r:id="rId12"/>
-    <hyperlink ref="D12" r:id="rId13"/>
-    <hyperlink ref="G12" r:id="rId14"/>
+    <hyperlink ref="G10" r:id="rId11"/>
+    <hyperlink ref="D11" r:id="rId12"/>
+    <hyperlink ref="G11" r:id="rId13"/>
+    <hyperlink ref="D12" r:id="rId14"/>
     <hyperlink ref="D13" r:id="rId15"/>
     <hyperlink ref="D14" r:id="rId16"/>
-    <hyperlink ref="D15" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
@@ -4109,7 +4134,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4121,174 +4146,174 @@
     </row>
     <row r="3" spans="1:8" ht="32" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="35" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B4" s="10" t="str">
         <f>IF(ABS(CAC_LTV!B7-7000)&lt;0.000001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="35" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="B5" s="10" t="str">
         <f>IF(ABS(CAC_LTV!C7-4000)&lt;0.000001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="35" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B6" s="10" t="str">
         <f>IF(ABS(CAC_LTV!B14-0.18*EXP(-0.4))&lt;0.000000001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="35" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="B7" s="10" t="str">
         <f>IF(ABS(CAC_LTV!B8-17398.8668944561)&lt;0.00001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="35" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="B8" s="10" t="str">
         <f>IF(ABS(Churn!D6-CAC_LTV!B8)&lt;0.00001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="35" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B9" s="10" t="str">
         <f>IF(ABS(TCO!B12-281000)&lt;0.00001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="35" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B10" s="10" t="str">
         <f>IF(ABS(TCO!C12-164000)&lt;0.00001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="35" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="B11" s="10" t="str">
         <f>IF(AND(ABS(SUM(TCO!B19:B23)-TCO!B12)&lt;0.00001,ABS(SUM(TCO!C19:C23)-TCO!C12)&lt;0.00001),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="35" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="B12" s="10" t="str">
         <f>IF(ABS(Sensitivity!E7+27000)&lt;0.00001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="35" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="B13" s="10" t="str">
         <f>IF(AND(Churn!B4&gt;Churn!B8,Churn!C4&lt;Churn!C8),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="35" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="B14" s="10" t="str">
         <f>IF(ABS(CAC_LTV!G18-5700/1.1)&lt;0.00001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="35" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B15" s="10" t="str">
         <f>IF(ABS(CAC_LTV!B24-CAC_LTV!B8*(1-CAC_LTV!B14))&lt;0.00001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="35" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B16" s="10" t="str">
         <f>IF(AND(Inputs!$B$16=4,Inputs!$B$25=7,Inputs!$B$21=0.3,Inputs!$B$5=5),"PASS","CHANGED")</f>
         <v>PASS</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="25" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>

</xml_diff>

<commit_message>
Finalize report without reference access dates or submission material
</commit_message>
<xml_diff>
--- a/deliverables/assignment1_models.xlsx
+++ b/deliverables/assignment1_models.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="272">
   <si>
     <t>Assignment 1 | Model guide and scope</t>
   </si>
@@ -77,10 +77,7 @@
     <t>Sources maps the official documentation to specific claims and records publication/revision dates. Licensing, staffing and hardware inputs are planning assumptions; procurement requires current entitlements and comparable quotations.</t>
   </si>
   <si>
-    <t>Readiness: see Checks. Cached values are included; open in Excel/LibreOffice to recalculate after changing inputs. External PNG/PDF/SVG figures represent the original baseline and do not auto-refresh.</t>
-  </si>
-  <si>
-    <t>Submission: student must review all reasoning and citations, add identification as required, complete VeriGuide and the institution’s Signed Declaration, attach authentic evidence and submit via Blackboard.</t>
+    <t>Model validation: see Checks. Cached values are included; open in Excel/LibreOffice to recalculate after changing inputs. External PNG/PDF/SVG figures represent the original baseline and do not auto-refresh.</t>
   </si>
   <si>
     <t>Inputs | All numbers are illustrative assumptions</t>
@@ -1679,7 +1676,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr defaultRowHeight="22" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="35.7109375" customWidth="1"/>
@@ -1918,30 +1915,8 @@
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
     </row>
-    <row r="34" spans="1:8" ht="25" customHeight="1">
-      <c r="A34" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-    </row>
-    <row r="35" spans="1:8" ht="25" customHeight="1">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
-    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="11">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A4:H5"/>
     <mergeCell ref="A7:H8"/>
@@ -1953,7 +1928,6 @@
     <mergeCell ref="A25:H26"/>
     <mergeCell ref="A28:H29"/>
     <mergeCell ref="A31:H32"/>
-    <mergeCell ref="A34:H35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
@@ -1980,7 +1954,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1992,366 +1966,366 @@
     </row>
     <row r="3" spans="1:8" ht="32" customHeight="1">
       <c r="A3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="32" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" s="5">
         <v>200</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="32" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5" s="5">
         <v>5</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="32" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6" s="5">
         <v>2026</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>23</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="32" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B7" s="5">
         <v>10</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="32" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" s="5">
         <v>70000</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="32" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B9" s="5">
         <v>70000</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="32" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B10" s="5">
         <v>30000</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="32" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B11" s="5">
         <v>6000</v>
       </c>
       <c r="C11" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="32" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B12" s="6">
         <v>0.05</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="32" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B13" s="6">
         <v>0.1</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="32" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B14" s="6">
         <v>0.18</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="32" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B15" s="5">
         <v>0.1</v>
       </c>
       <c r="C15" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>46</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="32" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B16" s="5">
         <v>4</v>
       </c>
       <c r="C16" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="32" customHeight="1">
       <c r="A17" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B17" s="5">
         <v>32000</v>
       </c>
       <c r="C17" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="32" customHeight="1">
       <c r="A18" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B18" s="5">
         <v>9000</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="32" customHeight="1">
       <c r="A19" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B19" s="5">
         <v>12000</v>
       </c>
       <c r="C19" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>57</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="32" customHeight="1">
       <c r="A20" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B20" s="5">
         <v>80000</v>
       </c>
       <c r="C20" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="32" customHeight="1">
       <c r="A21" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B21" s="5">
         <v>0.3</v>
       </c>
       <c r="C21" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>63</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="32" customHeight="1">
       <c r="A22" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B22" s="5">
         <v>7000</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="32" customHeight="1">
       <c r="A23" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B23" s="5">
         <v>5000</v>
       </c>
       <c r="C23" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D23" s="4" t="s">
         <v>68</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="32" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B24" s="5">
         <v>15000</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="32" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B25" s="5">
         <v>7</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="32" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B26" s="5">
         <v>8000</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="32" customHeight="1">
       <c r="A27" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B27" s="5">
         <v>14</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="32" customHeight="1">
       <c r="A28" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B28" s="5">
         <v>0.15</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -2472,7 +2446,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2484,18 +2458,18 @@
     </row>
     <row r="3" spans="1:8" ht="32" customHeight="1">
       <c r="A3" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>92</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="31" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B4" s="7">
         <f>Inputs!$B$8</f>
@@ -2508,7 +2482,7 @@
     </row>
     <row r="5" spans="1:8" ht="31" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B5" s="7">
         <f>0</f>
@@ -2521,7 +2495,7 @@
     </row>
     <row r="6" spans="1:8" ht="31" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B6" s="7">
         <f>B4-B5</f>
@@ -2534,7 +2508,7 @@
     </row>
     <row r="7" spans="1:8" ht="31" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B7" s="7">
         <f>B6/Inputs!$B$7</f>
@@ -2547,7 +2521,7 @@
     </row>
     <row r="8" spans="1:8" ht="31" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B8" s="7">
         <f>SUM(G18:G22)</f>
@@ -2560,7 +2534,7 @@
     </row>
     <row r="9" spans="1:8" ht="31" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B9" s="8">
         <f>B8/B7</f>
@@ -2573,7 +2547,7 @@
     </row>
     <row r="10" spans="1:8" ht="31" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B10" s="7">
         <f>B4/Inputs!$B$7</f>
@@ -2586,7 +2560,7 @@
     </row>
     <row r="11" spans="1:8" ht="31" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B11" s="8">
         <f>B8/B10</f>
@@ -2599,7 +2573,7 @@
     </row>
     <row r="13" spans="1:8" ht="22" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B13" s="8">
         <f>Inputs!$B$16</f>
@@ -2608,7 +2582,7 @@
     </row>
     <row r="14" spans="1:8" ht="22" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B14" s="9">
         <f>INDEX(Churn!B4:B8,MATCH(B13,Churn!A4:A8,0))</f>
@@ -2617,25 +2591,25 @@
     </row>
     <row r="17" spans="1:8" ht="32" customHeight="1">
       <c r="A17" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="C17" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="E17" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="F17" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="G17" s="3" t="s">
         <v>109</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="22" customHeight="1">
@@ -2785,7 +2759,7 @@
     </row>
     <row r="24" spans="1:8" ht="22" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B24" s="7">
         <f>B8*(1-B14)</f>
@@ -2794,7 +2768,7 @@
     </row>
     <row r="27" spans="1:8" ht="25" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -2816,7 +2790,7 @@
     </row>
     <row r="30" spans="1:8" ht="25" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -2864,7 +2838,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2876,22 +2850,22 @@
     </row>
     <row r="3" spans="1:8" ht="32" customHeight="1">
       <c r="A3" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>86</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="22" customHeight="1">
@@ -3021,7 +2995,7 @@
     </row>
     <row r="11" spans="1:8" ht="25" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -3043,7 +3017,7 @@
     </row>
     <row r="14" spans="1:8" ht="25" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -3093,7 +3067,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3105,21 +3079,21 @@
     </row>
     <row r="3" spans="1:8" ht="32" customHeight="1">
       <c r="A3" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>117</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="32" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B4" s="7">
         <f>Inputs!$B$17</f>
@@ -3130,12 +3104,12 @@
         <v>0</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="32" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B5" s="7">
         <f>Inputs!$B$18</f>
@@ -3146,12 +3120,12 @@
         <v>15000</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="32" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B6" s="7">
         <f>SUM(B4:B5)</f>
@@ -3162,12 +3136,12 @@
         <v>15000</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="32" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B7" s="7">
         <f>Inputs!$B$19</f>
@@ -3178,12 +3152,12 @@
         <v>16800</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="32" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B8" s="7">
         <f>Inputs!$B$20*Inputs!$B$21</f>
@@ -3194,12 +3168,12 @@
         <v>8000</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="32" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B9" s="7">
         <f>Inputs!$B$22</f>
@@ -3210,12 +3184,12 @@
         <v>0</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="32" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B10" s="7">
         <f>Inputs!$B$23</f>
@@ -3226,12 +3200,12 @@
         <v>5000</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="32" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B11" s="7">
         <f>SUM(B7:B10)</f>
@@ -3242,12 +3216,12 @@
         <v>29800</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="32" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B12" s="7">
         <f>B6+Inputs!$B$5*B11</f>
@@ -3258,12 +3232,12 @@
         <v>164000</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="22" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B14" s="7">
         <f>B12-C12</f>
@@ -3272,7 +3246,7 @@
     </row>
     <row r="15" spans="1:8" ht="22" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B15" s="9">
         <f>B14/B12</f>
@@ -3281,19 +3255,19 @@
     </row>
     <row r="18" spans="1:8" ht="32" customHeight="1">
       <c r="A18" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="D18" s="3" t="s">
+      <c r="E18" s="3" t="s">
         <v>140</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="22" customHeight="1">
@@ -3403,7 +3377,7 @@
     </row>
     <row r="26" spans="1:8" ht="25" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -3425,7 +3399,7 @@
     </row>
     <row r="29" spans="1:8" ht="25" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -3473,7 +3447,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3485,22 +3459,22 @@
     </row>
     <row r="3" spans="1:8" ht="32" customHeight="1">
       <c r="A3" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>149</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="22" customHeight="1">
@@ -3609,13 +3583,13 @@
     </row>
     <row r="10" spans="1:8" ht="32" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="22" customHeight="1">
@@ -3628,7 +3602,7 @@
         <v>16.75</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="22" customHeight="1">
@@ -3641,12 +3615,12 @@
         <v>11.75</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="25" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -3693,7 +3667,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3705,7 +3679,7 @@
     </row>
     <row r="49" spans="1:8" ht="25" customHeight="1">
       <c r="A49" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -3755,7 +3729,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3767,307 +3741,307 @@
     </row>
     <row r="3" spans="1:8" ht="32" customHeight="1">
       <c r="A3" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>162</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="95" customHeight="1">
       <c r="A4" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>168</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>169</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="95" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>175</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>176</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="95" customHeight="1">
       <c r="A6" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>182</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>183</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="95" customHeight="1">
       <c r="A7" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="H7" s="4" t="s">
         <v>191</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="95" customHeight="1">
       <c r="A8" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="F8" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>198</v>
-      </c>
       <c r="H8" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="95" customHeight="1">
       <c r="A9" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="F9" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="G9" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>204</v>
-      </c>
       <c r="H9" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="95" customHeight="1">
       <c r="A10" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="F10" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="G10" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="H10" s="4" t="s">
         <v>211</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="95" customHeight="1">
       <c r="A11" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="C11" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="E11" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="F11" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="F11" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="G11" s="4" t="s">
+      <c r="H11" s="4" t="s">
         <v>218</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="95" customHeight="1">
       <c r="A12" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C12" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="F12" s="4" t="s">
         <v>224</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>225</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="95" customHeight="1">
       <c r="A13" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="C13" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="F13" s="4" t="s">
         <v>231</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>232</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="95" customHeight="1">
       <c r="A14" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="C14" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="F14" s="4" t="s">
         <v>238</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>239</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="25" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -4134,7 +4108,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4146,174 +4120,174 @@
     </row>
     <row r="3" spans="1:8" ht="32" customHeight="1">
       <c r="A3" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>244</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="35" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B4" s="10" t="str">
         <f>IF(ABS(CAC_LTV!B7-7000)&lt;0.000001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="35" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B5" s="10" t="str">
         <f>IF(ABS(CAC_LTV!C7-4000)&lt;0.000001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="35" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B6" s="10" t="str">
         <f>IF(ABS(CAC_LTV!B14-0.18*EXP(-0.4))&lt;0.000000001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="35" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B7" s="10" t="str">
         <f>IF(ABS(CAC_LTV!B8-17398.8668944561)&lt;0.00001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="35" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B8" s="10" t="str">
         <f>IF(ABS(Churn!D6-CAC_LTV!B8)&lt;0.00001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="35" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B9" s="10" t="str">
         <f>IF(ABS(TCO!B12-281000)&lt;0.00001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="35" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B10" s="10" t="str">
         <f>IF(ABS(TCO!C12-164000)&lt;0.00001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="35" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B11" s="10" t="str">
         <f>IF(AND(ABS(SUM(TCO!B19:B23)-TCO!B12)&lt;0.00001,ABS(SUM(TCO!C19:C23)-TCO!C12)&lt;0.00001),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="35" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B12" s="10" t="str">
         <f>IF(ABS(Sensitivity!E7+27000)&lt;0.00001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="35" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B13" s="10" t="str">
         <f>IF(AND(Churn!B4&gt;Churn!B8,Churn!C4&lt;Churn!C8),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="35" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B14" s="10" t="str">
         <f>IF(ABS(CAC_LTV!G18-5700/1.1)&lt;0.00001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="35" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B15" s="10" t="str">
         <f>IF(ABS(CAC_LTV!B24-CAC_LTV!B8*(1-CAC_LTV!B14))&lt;0.00001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="35" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B16" s="10" t="str">
         <f>IF(AND(Inputs!$B$16=4,Inputs!$B$25=7,Inputs!$B$21=0.3,Inputs!$B$5=5),"PASS","CHANGED")</f>
         <v>PASS</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="25" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>

</xml_diff>